<commit_message>
se adecuan pruebas, se elimina comentarios neutros
</commit_message>
<xml_diff>
--- a/prueba01.xlsx
+++ b/prueba01.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae46519d9f6f6d4/2025/Curso Oracle ONE/Hackaton/testing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{84F742E9-2BAB-41B5-90D0-862F6F64B26F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF9AB94B-5380-43C3-85CC-001BC9066DF7}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{84F742E9-2BAB-41B5-90D0-862F6F64B26F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23E7A617-4306-441B-BB9A-E35F938708EA}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{D45572E8-3144-48DE-B926-C2FEC7453845}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{D45572E8-3144-48DE-B926-C2FEC7453845}"/>
   </bookViews>
   <sheets>
     <sheet name="positivos " sheetId="1" r:id="rId1"/>
     <sheet name="negativos" sheetId="2" r:id="rId2"/>
-    <sheet name="neutro" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="390">
   <si>
     <t>Está buenísimo, me encantó de una.</t>
   </si>
@@ -1197,390 +1196,6 @@
   </si>
   <si>
     <t>Horrible, una pérdida total.</t>
-  </si>
-  <si>
-    <t>Funciona como se espera.</t>
-  </si>
-  <si>
-    <t>Cumple lo básico, sin más.</t>
-  </si>
-  <si>
-    <t>Normal, nada fuera de lo común.</t>
-  </si>
-  <si>
-    <t>Está bien, sin destacar.</t>
-  </si>
-  <si>
-    <t>Resultado estándar, esperado.</t>
-  </si>
-  <si>
-    <t>Funciona, pero nada especial.</t>
-  </si>
-  <si>
-    <t>Todo correcto, sin sorpresas.</t>
-  </si>
-  <si>
-    <t>Es lo que promete.</t>
-  </si>
-  <si>
-    <t>Servicio normal, sin problemas.</t>
-  </si>
-  <si>
-    <t>Cumple, pero hasta ahí.</t>
-  </si>
-  <si>
-    <t>Está ok, nada más.</t>
-  </si>
-  <si>
-    <t>Funciona de manera regular.</t>
-  </si>
-  <si>
-    <t>Resultado promedio.</t>
-  </si>
-  <si>
-    <t>Nada que comentar, funciona.</t>
-  </si>
-  <si>
-    <t>Servicio estándar.</t>
-  </si>
-  <si>
-    <t>Correcto, sin destacar.</t>
-  </si>
-  <si>
-    <t>Funciona como corresponde.</t>
-  </si>
-  <si>
-    <t>Normalito, cumple.</t>
-  </si>
-  <si>
-    <t>Todo dentro de lo esperado.</t>
-  </si>
-  <si>
-    <t>Sin errores visibles.</t>
-  </si>
-  <si>
-    <t>Es funcional.</t>
-  </si>
-  <si>
-    <t>Servicio común y corriente.</t>
-  </si>
-  <si>
-    <t>Funciona sin mayores cambios.</t>
-  </si>
-  <si>
-    <t>Está aceptable.</t>
-  </si>
-  <si>
-    <t>Resultado normal.</t>
-  </si>
-  <si>
-    <t>Nada fuera de lo esperado.</t>
-  </si>
-  <si>
-    <t>Funciona igual que otros.</t>
-  </si>
-  <si>
-    <t>Es correcto.</t>
-  </si>
-  <si>
-    <t>Servicio básico.</t>
-  </si>
-  <si>
-    <t>Cumple su función.</t>
-  </si>
-  <si>
-    <t>Está bien hecho, sin destacar.</t>
-  </si>
-  <si>
-    <t>Funciona normalmente.</t>
-  </si>
-  <si>
-    <t>Todo ok, estándar.</t>
-  </si>
-  <si>
-    <t>Resultado neutro.</t>
-  </si>
-  <si>
-    <t>Nada especial que mencionar.</t>
-  </si>
-  <si>
-    <t>Servicio regular.</t>
-  </si>
-  <si>
-    <t>Cumple con lo mínimo.</t>
-  </si>
-  <si>
-    <t>Funciona sin fallas notorias.</t>
-  </si>
-  <si>
-    <t>Normal, nada raro.</t>
-  </si>
-  <si>
-    <t>Está correcto.</t>
-  </si>
-  <si>
-    <t>Servicio sin novedades.</t>
-  </si>
-  <si>
-    <t>Funciona como siempre.</t>
-  </si>
-  <si>
-    <t>Resultado esperado.</t>
-  </si>
-  <si>
-    <t>Todo normal.</t>
-  </si>
-  <si>
-    <t>Sin cambios relevantes.</t>
-  </si>
-  <si>
-    <t>Es funcional, nada más.</t>
-  </si>
-  <si>
-    <t>Cumple lo prometido.</t>
-  </si>
-  <si>
-    <t>Nada que destacar.</t>
-  </si>
-  <si>
-    <t>Funciona adecuadamente.</t>
-  </si>
-  <si>
-    <t>Está dentro de lo normal.</t>
-  </si>
-  <si>
-    <t>Correcto, sin comentarios.</t>
-  </si>
-  <si>
-    <t>Resultado común.</t>
-  </si>
-  <si>
-    <t>Funciona sin inconvenientes.</t>
-  </si>
-  <si>
-    <t>Todo en orden.</t>
-  </si>
-  <si>
-    <t>Servicio promedio.</t>
-  </si>
-  <si>
-    <t>Cumple, sin más.</t>
-  </si>
-  <si>
-    <t>Está bien, normal.</t>
-  </si>
-  <si>
-    <t>Funciona igual que antes.</t>
-  </si>
-  <si>
-    <t>Nada fuera de lo común.</t>
-  </si>
-  <si>
-    <t>Servicio correcto.</t>
-  </si>
-  <si>
-    <t>Resultado estándar.</t>
-  </si>
-  <si>
-    <t>Funciona según lo esperado.</t>
-  </si>
-  <si>
-    <t>Todo regular.</t>
-  </si>
-  <si>
-    <t>Es aceptable.</t>
-  </si>
-  <si>
-    <t>Funciona, punto.</t>
-  </si>
-  <si>
-    <t>Servicio simple.</t>
-  </si>
-  <si>
-    <t>Nada especial.</t>
-  </si>
-  <si>
-    <t>Resultado sin variaciones.</t>
-  </si>
-  <si>
-    <t>Está ok.</t>
-  </si>
-  <si>
-    <t>Cumple lo básico.</t>
-  </si>
-  <si>
-    <t>Servicio funcional.</t>
-  </si>
-  <si>
-    <t>Funciona normal.</t>
-  </si>
-  <si>
-    <t>Resultado habitual.</t>
-  </si>
-  <si>
-    <t>Todo correcto.</t>
-  </si>
-  <si>
-    <t>Sin observaciones.</t>
-  </si>
-  <si>
-    <t>Servicio común.</t>
-  </si>
-  <si>
-    <t>Normalito.</t>
-  </si>
-  <si>
-    <t>Nada relevante.</t>
-  </si>
-  <si>
-    <t>Está dentro del promedio.</t>
-  </si>
-  <si>
-    <t>Resultado sin cambios.</t>
-  </si>
-  <si>
-    <t>Funciona correctamente.</t>
-  </si>
-  <si>
-    <t>Cumple sin destacar.</t>
-  </si>
-  <si>
-    <t>Todo normal, ok.</t>
-  </si>
-  <si>
-    <t>Nada fuera de lugar.</t>
-  </si>
-  <si>
-    <t>Funciona bien, normal.</t>
-  </si>
-  <si>
-    <t>Servicio sin problemas.</t>
-  </si>
-  <si>
-    <t>Funciona tal cual.</t>
-  </si>
-  <si>
-    <t>Está bien, promedio.</t>
-  </si>
-  <si>
-    <t>Nada que decir.</t>
-  </si>
-  <si>
-    <t>Cumple lo justo.</t>
-  </si>
-  <si>
-    <t>Servicio neutro.</t>
-  </si>
-  <si>
-    <t>Funciona sin novedad.</t>
-  </si>
-  <si>
-    <t>Resultado común y corriente.</t>
-  </si>
-  <si>
-    <t>Todo en regla.</t>
-  </si>
-  <si>
-    <t>Normal.</t>
-  </si>
-  <si>
-    <t>Funciona correctamente, estándar.</t>
-  </si>
-  <si>
-    <t>Cumple lo mínimo esperado.</t>
-  </si>
-  <si>
-    <t>Está bien, nada más.</t>
-  </si>
-  <si>
-    <t>Funciona sin cambios.</t>
-  </si>
-  <si>
-    <t>Todo correcto, normal.</t>
-  </si>
-  <si>
-    <t>Nada destacable.</t>
-  </si>
-  <si>
-    <t>Funciona y ya.</t>
-  </si>
-  <si>
-    <t>Está dentro de lo esperado.</t>
-  </si>
-  <si>
-    <t>Funciona bien, sin más.</t>
-  </si>
-  <si>
-    <t>Todo normal, correcto.</t>
-  </si>
-  <si>
-    <t>Cumple con su función.</t>
-  </si>
-  <si>
-    <t>Nada fuera de lo normal.</t>
-  </si>
-  <si>
-    <t>Resultado aceptable.</t>
-  </si>
-  <si>
-    <t>Está ok, cumple.</t>
-  </si>
-  <si>
-    <t>Todo dentro de lo normal.</t>
-  </si>
-  <si>
-    <t>Nada especial que decir.</t>
-  </si>
-  <si>
-    <t>Está bien, normalito.</t>
-  </si>
-  <si>
-    <t>Funciona sin errores aparentes.</t>
-  </si>
-  <si>
-    <t>Funciona como debería.</t>
-  </si>
-  <si>
-    <t>Está correcto, sin más.</t>
-  </si>
-  <si>
-    <t>Funciona bien, estándar.</t>
-  </si>
-  <si>
-    <t>Todo correcto, promedio.</t>
-  </si>
-  <si>
-    <t>Cumple su propósito.</t>
-  </si>
-  <si>
-    <t>Está ok, normal.</t>
-  </si>
-  <si>
-    <t>Resultado sin sorpresas.</t>
-  </si>
-  <si>
-    <t>Funciona correctamente, normal.</t>
-  </si>
-  <si>
-    <t>Cumple, sin comentarios.</t>
-  </si>
-  <si>
-    <t>Funciona como esperado.</t>
-  </si>
-  <si>
-    <t>Funciona sin problemas.</t>
-  </si>
-  <si>
-    <t>Todo normal, estándar.</t>
-  </si>
-  <si>
-    <t>Funciona bien, normalito.</t>
-  </si>
-  <si>
-    <t>Todo dentro del promedio.</t>
-  </si>
-  <si>
-    <t>Funciona correctamente, promedio.</t>
   </si>
   <si>
     <t>#</t>
@@ -1949,13 +1564,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>515</v>
+        <v>387</v>
       </c>
       <c r="B1" t="s">
-        <v>516</v>
+        <v>388</v>
       </c>
       <c r="C1" t="s">
-        <v>517</v>
+        <v>389</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -4176,13 +3791,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>515</v>
+        <v>387</v>
       </c>
       <c r="B1" t="s">
-        <v>516</v>
+        <v>388</v>
       </c>
       <c r="C1" t="s">
-        <v>517</v>
+        <v>389</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -4193,7 +3808,7 @@
         <v>193</v>
       </c>
       <c r="C2">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -4204,7 +3819,7 @@
         <v>194</v>
       </c>
       <c r="C3">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -4215,7 +3830,7 @@
         <v>195</v>
       </c>
       <c r="C4">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4226,7 +3841,7 @@
         <v>196</v>
       </c>
       <c r="C5">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4237,7 +3852,7 @@
         <v>197</v>
       </c>
       <c r="C6">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4248,7 +3863,7 @@
         <v>198</v>
       </c>
       <c r="C7">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4259,7 +3874,7 @@
         <v>199</v>
       </c>
       <c r="C8">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -4270,7 +3885,7 @@
         <v>200</v>
       </c>
       <c r="C9">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -4281,7 +3896,7 @@
         <v>201</v>
       </c>
       <c r="C10">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -4292,7 +3907,7 @@
         <v>202</v>
       </c>
       <c r="C11">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -4303,7 +3918,7 @@
         <v>203</v>
       </c>
       <c r="C12">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -4314,7 +3929,7 @@
         <v>204</v>
       </c>
       <c r="C13">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -4325,7 +3940,7 @@
         <v>205</v>
       </c>
       <c r="C14">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -4336,7 +3951,7 @@
         <v>206</v>
       </c>
       <c r="C15">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -4347,7 +3962,7 @@
         <v>207</v>
       </c>
       <c r="C16">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -4358,7 +3973,7 @@
         <v>208</v>
       </c>
       <c r="C17">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -4369,7 +3984,7 @@
         <v>209</v>
       </c>
       <c r="C18">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -4380,7 +3995,7 @@
         <v>210</v>
       </c>
       <c r="C19">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -4391,7 +4006,7 @@
         <v>211</v>
       </c>
       <c r="C20">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -4402,7 +4017,7 @@
         <v>212</v>
       </c>
       <c r="C21">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -4413,7 +4028,7 @@
         <v>213</v>
       </c>
       <c r="C22">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -4424,7 +4039,7 @@
         <v>214</v>
       </c>
       <c r="C23">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -4435,7 +4050,7 @@
         <v>215</v>
       </c>
       <c r="C24">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -4446,7 +4061,7 @@
         <v>216</v>
       </c>
       <c r="C25">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -4457,7 +4072,7 @@
         <v>217</v>
       </c>
       <c r="C26">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -4468,7 +4083,7 @@
         <v>218</v>
       </c>
       <c r="C27">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -4479,7 +4094,7 @@
         <v>219</v>
       </c>
       <c r="C28">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -4490,7 +4105,7 @@
         <v>220</v>
       </c>
       <c r="C29">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -4501,7 +4116,7 @@
         <v>221</v>
       </c>
       <c r="C30">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -4512,7 +4127,7 @@
         <v>222</v>
       </c>
       <c r="C31">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -4523,7 +4138,7 @@
         <v>223</v>
       </c>
       <c r="C32">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -4534,7 +4149,7 @@
         <v>224</v>
       </c>
       <c r="C33">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -4545,7 +4160,7 @@
         <v>225</v>
       </c>
       <c r="C34">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -4556,7 +4171,7 @@
         <v>226</v>
       </c>
       <c r="C35">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -4567,7 +4182,7 @@
         <v>227</v>
       </c>
       <c r="C36">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -4578,7 +4193,7 @@
         <v>228</v>
       </c>
       <c r="C37">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -4589,7 +4204,7 @@
         <v>229</v>
       </c>
       <c r="C38">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -4600,7 +4215,7 @@
         <v>230</v>
       </c>
       <c r="C39">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -4611,7 +4226,7 @@
         <v>231</v>
       </c>
       <c r="C40">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -4622,7 +4237,7 @@
         <v>232</v>
       </c>
       <c r="C41">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -4633,7 +4248,7 @@
         <v>233</v>
       </c>
       <c r="C42">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -4644,7 +4259,7 @@
         <v>234</v>
       </c>
       <c r="C43">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -4655,7 +4270,7 @@
         <v>235</v>
       </c>
       <c r="C44">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -4666,7 +4281,7 @@
         <v>236</v>
       </c>
       <c r="C45">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -4677,7 +4292,7 @@
         <v>237</v>
       </c>
       <c r="C46">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -4688,7 +4303,7 @@
         <v>238</v>
       </c>
       <c r="C47">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -4699,7 +4314,7 @@
         <v>239</v>
       </c>
       <c r="C48">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -4710,7 +4325,7 @@
         <v>240</v>
       </c>
       <c r="C49">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -4721,7 +4336,7 @@
         <v>241</v>
       </c>
       <c r="C50">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -4732,7 +4347,7 @@
         <v>242</v>
       </c>
       <c r="C51">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -4743,7 +4358,7 @@
         <v>243</v>
       </c>
       <c r="C52">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -4754,7 +4369,7 @@
         <v>244</v>
       </c>
       <c r="C53">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -4765,7 +4380,7 @@
         <v>245</v>
       </c>
       <c r="C54">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -4776,7 +4391,7 @@
         <v>246</v>
       </c>
       <c r="C55">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -4787,7 +4402,7 @@
         <v>247</v>
       </c>
       <c r="C56">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -4798,7 +4413,7 @@
         <v>248</v>
       </c>
       <c r="C57">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -4809,7 +4424,7 @@
         <v>249</v>
       </c>
       <c r="C58">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -4820,7 +4435,7 @@
         <v>250</v>
       </c>
       <c r="C59">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -4831,7 +4446,7 @@
         <v>251</v>
       </c>
       <c r="C60">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -4842,7 +4457,7 @@
         <v>252</v>
       </c>
       <c r="C61">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -4853,7 +4468,7 @@
         <v>253</v>
       </c>
       <c r="C62">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -4864,7 +4479,7 @@
         <v>254</v>
       </c>
       <c r="C63">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -4875,7 +4490,7 @@
         <v>255</v>
       </c>
       <c r="C64">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -4886,7 +4501,7 @@
         <v>256</v>
       </c>
       <c r="C65">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
@@ -4897,7 +4512,7 @@
         <v>257</v>
       </c>
       <c r="C66">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -4908,7 +4523,7 @@
         <v>258</v>
       </c>
       <c r="C67">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
@@ -4919,7 +4534,7 @@
         <v>259</v>
       </c>
       <c r="C68">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
@@ -4930,7 +4545,7 @@
         <v>260</v>
       </c>
       <c r="C69">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
@@ -4941,7 +4556,7 @@
         <v>261</v>
       </c>
       <c r="C70">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
@@ -4952,7 +4567,7 @@
         <v>262</v>
       </c>
       <c r="C71">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
@@ -4963,7 +4578,7 @@
         <v>263</v>
       </c>
       <c r="C72">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
@@ -4974,7 +4589,7 @@
         <v>264</v>
       </c>
       <c r="C73">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
@@ -4985,7 +4600,7 @@
         <v>265</v>
       </c>
       <c r="C74">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
@@ -4996,7 +4611,7 @@
         <v>266</v>
       </c>
       <c r="C75">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
@@ -5007,7 +4622,7 @@
         <v>267</v>
       </c>
       <c r="C76">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
@@ -5018,7 +4633,7 @@
         <v>268</v>
       </c>
       <c r="C77">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
@@ -5029,7 +4644,7 @@
         <v>269</v>
       </c>
       <c r="C78">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
@@ -5040,7 +4655,7 @@
         <v>270</v>
       </c>
       <c r="C79">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
@@ -5051,7 +4666,7 @@
         <v>271</v>
       </c>
       <c r="C80">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
@@ -5062,7 +4677,7 @@
         <v>272</v>
       </c>
       <c r="C81">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
@@ -5073,7 +4688,7 @@
         <v>273</v>
       </c>
       <c r="C82">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
@@ -5084,7 +4699,7 @@
         <v>274</v>
       </c>
       <c r="C83">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -5095,7 +4710,7 @@
         <v>275</v>
       </c>
       <c r="C84">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -5106,7 +4721,7 @@
         <v>276</v>
       </c>
       <c r="C85">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -5117,7 +4732,7 @@
         <v>277</v>
       </c>
       <c r="C86">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -5128,7 +4743,7 @@
         <v>278</v>
       </c>
       <c r="C87">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
@@ -5139,7 +4754,7 @@
         <v>279</v>
       </c>
       <c r="C88">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
@@ -5150,7 +4765,7 @@
         <v>280</v>
       </c>
       <c r="C89">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
@@ -5161,7 +4776,7 @@
         <v>281</v>
       </c>
       <c r="C90">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
@@ -5172,7 +4787,7 @@
         <v>282</v>
       </c>
       <c r="C91">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
@@ -5183,7 +4798,7 @@
         <v>283</v>
       </c>
       <c r="C92">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
@@ -5194,7 +4809,7 @@
         <v>284</v>
       </c>
       <c r="C93">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
@@ -5205,7 +4820,7 @@
         <v>285</v>
       </c>
       <c r="C94">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
@@ -5216,7 +4831,7 @@
         <v>286</v>
       </c>
       <c r="C95">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
@@ -5227,7 +4842,7 @@
         <v>287</v>
       </c>
       <c r="C96">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
@@ -5238,7 +4853,7 @@
         <v>288</v>
       </c>
       <c r="C97">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
@@ -5249,7 +4864,7 @@
         <v>289</v>
       </c>
       <c r="C98">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
@@ -5260,7 +4875,7 @@
         <v>290</v>
       </c>
       <c r="C99">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
@@ -5271,7 +4886,7 @@
         <v>291</v>
       </c>
       <c r="C100">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
@@ -5282,7 +4897,7 @@
         <v>292</v>
       </c>
       <c r="C101">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
@@ -5293,7 +4908,7 @@
         <v>293</v>
       </c>
       <c r="C102">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
@@ -5304,7 +4919,7 @@
         <v>294</v>
       </c>
       <c r="C103">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
@@ -5315,7 +4930,7 @@
         <v>295</v>
       </c>
       <c r="C104">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
@@ -5326,7 +4941,7 @@
         <v>296</v>
       </c>
       <c r="C105">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
@@ -5337,7 +4952,7 @@
         <v>297</v>
       </c>
       <c r="C106">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
@@ -5348,7 +4963,7 @@
         <v>298</v>
       </c>
       <c r="C107">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
@@ -5359,7 +4974,7 @@
         <v>299</v>
       </c>
       <c r="C108">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
@@ -5370,7 +4985,7 @@
         <v>300</v>
       </c>
       <c r="C109">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
@@ -5381,7 +4996,7 @@
         <v>301</v>
       </c>
       <c r="C110">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
@@ -5392,7 +5007,7 @@
         <v>302</v>
       </c>
       <c r="C111">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
@@ -5403,7 +5018,7 @@
         <v>303</v>
       </c>
       <c r="C112">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
@@ -5414,7 +5029,7 @@
         <v>304</v>
       </c>
       <c r="C113">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
@@ -5425,7 +5040,7 @@
         <v>305</v>
       </c>
       <c r="C114">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
@@ -5436,7 +5051,7 @@
         <v>306</v>
       </c>
       <c r="C115">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
@@ -5447,7 +5062,7 @@
         <v>307</v>
       </c>
       <c r="C116">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
@@ -5458,7 +5073,7 @@
         <v>308</v>
       </c>
       <c r="C117">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
@@ -5469,7 +5084,7 @@
         <v>309</v>
       </c>
       <c r="C118">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
@@ -5480,7 +5095,7 @@
         <v>310</v>
       </c>
       <c r="C119">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
@@ -5491,7 +5106,7 @@
         <v>311</v>
       </c>
       <c r="C120">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
@@ -5502,7 +5117,7 @@
         <v>312</v>
       </c>
       <c r="C121">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
@@ -5513,7 +5128,7 @@
         <v>313</v>
       </c>
       <c r="C122">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
@@ -5524,7 +5139,7 @@
         <v>314</v>
       </c>
       <c r="C123">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
@@ -5535,7 +5150,7 @@
         <v>315</v>
       </c>
       <c r="C124">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
@@ -5546,7 +5161,7 @@
         <v>316</v>
       </c>
       <c r="C125">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
@@ -5557,7 +5172,7 @@
         <v>317</v>
       </c>
       <c r="C126">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
@@ -5568,7 +5183,7 @@
         <v>318</v>
       </c>
       <c r="C127">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
@@ -5579,7 +5194,7 @@
         <v>319</v>
       </c>
       <c r="C128">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
@@ -5590,7 +5205,7 @@
         <v>320</v>
       </c>
       <c r="C129">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
@@ -5601,7 +5216,7 @@
         <v>321</v>
       </c>
       <c r="C130">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
@@ -5612,7 +5227,7 @@
         <v>229</v>
       </c>
       <c r="C131">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -5623,7 +5238,7 @@
         <v>322</v>
       </c>
       <c r="C132">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
@@ -5634,7 +5249,7 @@
         <v>323</v>
       </c>
       <c r="C133">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
@@ -5645,7 +5260,7 @@
         <v>324</v>
       </c>
       <c r="C134">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
@@ -5656,7 +5271,7 @@
         <v>325</v>
       </c>
       <c r="C135">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
@@ -5667,7 +5282,7 @@
         <v>326</v>
       </c>
       <c r="C136">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
@@ -5678,7 +5293,7 @@
         <v>327</v>
       </c>
       <c r="C137">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
@@ -5689,7 +5304,7 @@
         <v>328</v>
       </c>
       <c r="C138">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
@@ -5700,7 +5315,7 @@
         <v>329</v>
       </c>
       <c r="C139">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
@@ -5711,7 +5326,7 @@
         <v>330</v>
       </c>
       <c r="C140">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
@@ -5722,7 +5337,7 @@
         <v>331</v>
       </c>
       <c r="C141">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
@@ -5733,7 +5348,7 @@
         <v>332</v>
       </c>
       <c r="C142">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
@@ -5744,7 +5359,7 @@
         <v>333</v>
       </c>
       <c r="C143">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
@@ -5755,7 +5370,7 @@
         <v>334</v>
       </c>
       <c r="C144">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
@@ -5766,7 +5381,7 @@
         <v>335</v>
       </c>
       <c r="C145">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
@@ -5777,7 +5392,7 @@
         <v>336</v>
       </c>
       <c r="C146">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
@@ -5788,7 +5403,7 @@
         <v>337</v>
       </c>
       <c r="C147">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
@@ -5799,7 +5414,7 @@
         <v>338</v>
       </c>
       <c r="C148">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
@@ -5810,7 +5425,7 @@
         <v>339</v>
       </c>
       <c r="C149">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
@@ -5821,7 +5436,7 @@
         <v>340</v>
       </c>
       <c r="C150">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
@@ -5832,7 +5447,7 @@
         <v>341</v>
       </c>
       <c r="C151">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
@@ -5843,7 +5458,7 @@
         <v>297</v>
       </c>
       <c r="C152">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
@@ -5854,7 +5469,7 @@
         <v>342</v>
       </c>
       <c r="C153">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
@@ -5865,7 +5480,7 @@
         <v>343</v>
       </c>
       <c r="C154">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
@@ -5876,7 +5491,7 @@
         <v>344</v>
       </c>
       <c r="C155">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
@@ -5887,7 +5502,7 @@
         <v>345</v>
       </c>
       <c r="C156">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
@@ -5898,7 +5513,7 @@
         <v>234</v>
       </c>
       <c r="C157">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
@@ -5909,7 +5524,7 @@
         <v>346</v>
       </c>
       <c r="C158">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
@@ -5920,7 +5535,7 @@
         <v>347</v>
       </c>
       <c r="C159">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
@@ -5931,7 +5546,7 @@
         <v>348</v>
       </c>
       <c r="C160">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
@@ -5942,7 +5557,7 @@
         <v>349</v>
       </c>
       <c r="C161">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
@@ -5953,7 +5568,7 @@
         <v>350</v>
       </c>
       <c r="C162">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
@@ -5964,7 +5579,7 @@
         <v>351</v>
       </c>
       <c r="C163">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
@@ -5975,7 +5590,7 @@
         <v>352</v>
       </c>
       <c r="C164">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
@@ -5986,7 +5601,7 @@
         <v>353</v>
       </c>
       <c r="C165">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
@@ -5997,7 +5612,7 @@
         <v>354</v>
       </c>
       <c r="C166">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
@@ -6008,7 +5623,7 @@
         <v>355</v>
       </c>
       <c r="C167">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
@@ -6019,7 +5634,7 @@
         <v>356</v>
       </c>
       <c r="C168">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
@@ -6030,7 +5645,7 @@
         <v>357</v>
       </c>
       <c r="C169">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
@@ -6041,7 +5656,7 @@
         <v>358</v>
       </c>
       <c r="C170">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
@@ -6052,7 +5667,7 @@
         <v>359</v>
       </c>
       <c r="C171">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
@@ -6063,7 +5678,7 @@
         <v>360</v>
       </c>
       <c r="C172">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
@@ -6074,7 +5689,7 @@
         <v>361</v>
       </c>
       <c r="C173">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
@@ -6085,7 +5700,7 @@
         <v>362</v>
       </c>
       <c r="C174">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
@@ -6096,7 +5711,7 @@
         <v>363</v>
       </c>
       <c r="C175">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
@@ -6107,7 +5722,7 @@
         <v>364</v>
       </c>
       <c r="C176">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
@@ -6118,7 +5733,7 @@
         <v>365</v>
       </c>
       <c r="C177">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
@@ -6129,7 +5744,7 @@
         <v>366</v>
       </c>
       <c r="C178">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
@@ -6140,7 +5755,7 @@
         <v>310</v>
       </c>
       <c r="C179">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
@@ -6151,7 +5766,7 @@
         <v>367</v>
       </c>
       <c r="C180">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
@@ -6162,7 +5777,7 @@
         <v>368</v>
       </c>
       <c r="C181">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
@@ -6173,7 +5788,7 @@
         <v>369</v>
       </c>
       <c r="C182">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
@@ -6184,7 +5799,7 @@
         <v>370</v>
       </c>
       <c r="C183">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
@@ -6195,7 +5810,7 @@
         <v>371</v>
       </c>
       <c r="C184">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
@@ -6206,7 +5821,7 @@
         <v>372</v>
       </c>
       <c r="C185">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
@@ -6217,7 +5832,7 @@
         <v>373</v>
       </c>
       <c r="C186">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
@@ -6228,7 +5843,7 @@
         <v>303</v>
       </c>
       <c r="C187">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
@@ -6239,7 +5854,7 @@
         <v>374</v>
       </c>
       <c r="C188">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
@@ -6250,7 +5865,7 @@
         <v>375</v>
       </c>
       <c r="C189">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
@@ -6261,7 +5876,7 @@
         <v>376</v>
       </c>
       <c r="C190">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
@@ -6272,7 +5887,7 @@
         <v>377</v>
       </c>
       <c r="C191">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
@@ -6283,7 +5898,7 @@
         <v>378</v>
       </c>
       <c r="C192">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
@@ -6294,7 +5909,7 @@
         <v>379</v>
       </c>
       <c r="C193">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
@@ -6305,7 +5920,7 @@
         <v>380</v>
       </c>
       <c r="C194">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
@@ -6316,7 +5931,7 @@
         <v>381</v>
       </c>
       <c r="C195">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
@@ -6327,7 +5942,7 @@
         <v>382</v>
       </c>
       <c r="C196">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
@@ -6338,7 +5953,7 @@
         <v>383</v>
       </c>
       <c r="C197">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
@@ -6349,7 +5964,7 @@
         <v>327</v>
       </c>
       <c r="C198">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
@@ -6360,7 +5975,7 @@
         <v>384</v>
       </c>
       <c r="C199">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
@@ -6371,7 +5986,7 @@
         <v>385</v>
       </c>
       <c r="C200">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
@@ -6382,7 +5997,7 @@
         <v>386</v>
       </c>
       <c r="C201">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -6391,2231 +6006,4 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89AEBB4C-B1CF-491F-944E-AF4D088BC9A5}">
-  <dimension ref="A1:C201"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="33.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>515</v>
-      </c>
-      <c r="B1" t="s">
-        <v>516</v>
-      </c>
-      <c r="C1" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>387</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>388</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>389</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>390</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>391</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>392</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>393</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>394</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>395</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>396</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>397</v>
-      </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>398</v>
-      </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>399</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>400</v>
-      </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>401</v>
-      </c>
-      <c r="C16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>402</v>
-      </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="s">
-        <v>403</v>
-      </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" t="s">
-        <v>404</v>
-      </c>
-      <c r="C19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="s">
-        <v>405</v>
-      </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="s">
-        <v>406</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="s">
-        <v>407</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="s">
-        <v>408</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" t="s">
-        <v>409</v>
-      </c>
-      <c r="C24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" t="s">
-        <v>410</v>
-      </c>
-      <c r="C25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="s">
-        <v>411</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" t="s">
-        <v>412</v>
-      </c>
-      <c r="C27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28" t="s">
-        <v>413</v>
-      </c>
-      <c r="C28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>28</v>
-      </c>
-      <c r="B29" t="s">
-        <v>414</v>
-      </c>
-      <c r="C29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>29</v>
-      </c>
-      <c r="B30" t="s">
-        <v>415</v>
-      </c>
-      <c r="C30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>30</v>
-      </c>
-      <c r="B31" t="s">
-        <v>416</v>
-      </c>
-      <c r="C31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>31</v>
-      </c>
-      <c r="B32" t="s">
-        <v>417</v>
-      </c>
-      <c r="C32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>32</v>
-      </c>
-      <c r="B33" t="s">
-        <v>418</v>
-      </c>
-      <c r="C33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>33</v>
-      </c>
-      <c r="B34" t="s">
-        <v>419</v>
-      </c>
-      <c r="C34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <v>34</v>
-      </c>
-      <c r="B35" t="s">
-        <v>420</v>
-      </c>
-      <c r="C35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>35</v>
-      </c>
-      <c r="B36" t="s">
-        <v>421</v>
-      </c>
-      <c r="C36">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <v>36</v>
-      </c>
-      <c r="B37" t="s">
-        <v>422</v>
-      </c>
-      <c r="C37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <v>37</v>
-      </c>
-      <c r="B38" t="s">
-        <v>423</v>
-      </c>
-      <c r="C38">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <v>38</v>
-      </c>
-      <c r="B39" t="s">
-        <v>424</v>
-      </c>
-      <c r="C39">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40">
-        <v>39</v>
-      </c>
-      <c r="B40" t="s">
-        <v>425</v>
-      </c>
-      <c r="C40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41">
-        <v>40</v>
-      </c>
-      <c r="B41" t="s">
-        <v>426</v>
-      </c>
-      <c r="C41">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42">
-        <v>41</v>
-      </c>
-      <c r="B42" t="s">
-        <v>427</v>
-      </c>
-      <c r="C42">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43">
-        <v>42</v>
-      </c>
-      <c r="B43" t="s">
-        <v>428</v>
-      </c>
-      <c r="C43">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44">
-        <v>43</v>
-      </c>
-      <c r="B44" t="s">
-        <v>429</v>
-      </c>
-      <c r="C44">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <v>44</v>
-      </c>
-      <c r="B45" t="s">
-        <v>430</v>
-      </c>
-      <c r="C45">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46">
-        <v>45</v>
-      </c>
-      <c r="B46" t="s">
-        <v>431</v>
-      </c>
-      <c r="C46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47">
-        <v>46</v>
-      </c>
-      <c r="B47" t="s">
-        <v>432</v>
-      </c>
-      <c r="C47">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48">
-        <v>47</v>
-      </c>
-      <c r="B48" t="s">
-        <v>433</v>
-      </c>
-      <c r="C48">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49">
-        <v>48</v>
-      </c>
-      <c r="B49" t="s">
-        <v>401</v>
-      </c>
-      <c r="C49">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50">
-        <v>49</v>
-      </c>
-      <c r="B50" t="s">
-        <v>434</v>
-      </c>
-      <c r="C50">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51">
-        <v>50</v>
-      </c>
-      <c r="B51" t="s">
-        <v>435</v>
-      </c>
-      <c r="C51">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52">
-        <v>51</v>
-      </c>
-      <c r="B52" t="s">
-        <v>436</v>
-      </c>
-      <c r="C52">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53">
-        <v>52</v>
-      </c>
-      <c r="B53" t="s">
-        <v>437</v>
-      </c>
-      <c r="C53">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54">
-        <v>53</v>
-      </c>
-      <c r="B54" t="s">
-        <v>438</v>
-      </c>
-      <c r="C54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55">
-        <v>54</v>
-      </c>
-      <c r="B55" t="s">
-        <v>439</v>
-      </c>
-      <c r="C55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56">
-        <v>55</v>
-      </c>
-      <c r="B56" t="s">
-        <v>440</v>
-      </c>
-      <c r="C56">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57">
-        <v>56</v>
-      </c>
-      <c r="B57" t="s">
-        <v>441</v>
-      </c>
-      <c r="C57">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58">
-        <v>57</v>
-      </c>
-      <c r="B58" t="s">
-        <v>442</v>
-      </c>
-      <c r="C58">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59">
-        <v>58</v>
-      </c>
-      <c r="B59" t="s">
-        <v>443</v>
-      </c>
-      <c r="C59">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60">
-        <v>59</v>
-      </c>
-      <c r="B60" t="s">
-        <v>444</v>
-      </c>
-      <c r="C60">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61">
-        <v>60</v>
-      </c>
-      <c r="B61" t="s">
-        <v>445</v>
-      </c>
-      <c r="C61">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62">
-        <v>61</v>
-      </c>
-      <c r="B62" t="s">
-        <v>446</v>
-      </c>
-      <c r="C62">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63">
-        <v>62</v>
-      </c>
-      <c r="B63" t="s">
-        <v>447</v>
-      </c>
-      <c r="C63">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64">
-        <v>63</v>
-      </c>
-      <c r="B64" t="s">
-        <v>448</v>
-      </c>
-      <c r="C64">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65">
-        <v>64</v>
-      </c>
-      <c r="B65" t="s">
-        <v>449</v>
-      </c>
-      <c r="C65">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66">
-        <v>65</v>
-      </c>
-      <c r="B66" t="s">
-        <v>450</v>
-      </c>
-      <c r="C66">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A67">
-        <v>66</v>
-      </c>
-      <c r="B67" t="s">
-        <v>451</v>
-      </c>
-      <c r="C67">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A68">
-        <v>67</v>
-      </c>
-      <c r="B68" t="s">
-        <v>452</v>
-      </c>
-      <c r="C68">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A69">
-        <v>68</v>
-      </c>
-      <c r="B69" t="s">
-        <v>453</v>
-      </c>
-      <c r="C69">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A70">
-        <v>69</v>
-      </c>
-      <c r="B70" t="s">
-        <v>454</v>
-      </c>
-      <c r="C70">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A71">
-        <v>70</v>
-      </c>
-      <c r="B71" t="s">
-        <v>455</v>
-      </c>
-      <c r="C71">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A72">
-        <v>71</v>
-      </c>
-      <c r="B72" t="s">
-        <v>456</v>
-      </c>
-      <c r="C72">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A73">
-        <v>72</v>
-      </c>
-      <c r="B73" t="s">
-        <v>457</v>
-      </c>
-      <c r="C73">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A74">
-        <v>73</v>
-      </c>
-      <c r="B74" t="s">
-        <v>458</v>
-      </c>
-      <c r="C74">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A75">
-        <v>74</v>
-      </c>
-      <c r="B75" t="s">
-        <v>459</v>
-      </c>
-      <c r="C75">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A76">
-        <v>75</v>
-      </c>
-      <c r="B76" t="s">
-        <v>460</v>
-      </c>
-      <c r="C76">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A77">
-        <v>76</v>
-      </c>
-      <c r="B77" t="s">
-        <v>461</v>
-      </c>
-      <c r="C77">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A78">
-        <v>77</v>
-      </c>
-      <c r="B78" t="s">
-        <v>462</v>
-      </c>
-      <c r="C78">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A79">
-        <v>78</v>
-      </c>
-      <c r="B79" t="s">
-        <v>403</v>
-      </c>
-      <c r="C79">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A80">
-        <v>79</v>
-      </c>
-      <c r="B80" t="s">
-        <v>463</v>
-      </c>
-      <c r="C80">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A81">
-        <v>80</v>
-      </c>
-      <c r="B81" t="s">
-        <v>464</v>
-      </c>
-      <c r="C81">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A82">
-        <v>81</v>
-      </c>
-      <c r="B82" t="s">
-        <v>465</v>
-      </c>
-      <c r="C82">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A83">
-        <v>82</v>
-      </c>
-      <c r="B83" t="s">
-        <v>422</v>
-      </c>
-      <c r="C83">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A84">
-        <v>83</v>
-      </c>
-      <c r="B84" t="s">
-        <v>466</v>
-      </c>
-      <c r="C84">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A85">
-        <v>84</v>
-      </c>
-      <c r="B85" t="s">
-        <v>467</v>
-      </c>
-      <c r="C85">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A86">
-        <v>85</v>
-      </c>
-      <c r="B86" t="s">
-        <v>468</v>
-      </c>
-      <c r="C86">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A87">
-        <v>86</v>
-      </c>
-      <c r="B87" t="s">
-        <v>469</v>
-      </c>
-      <c r="C87">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A88">
-        <v>87</v>
-      </c>
-      <c r="B88" t="s">
-        <v>401</v>
-      </c>
-      <c r="C88">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A89">
-        <v>88</v>
-      </c>
-      <c r="B89" t="s">
-        <v>470</v>
-      </c>
-      <c r="C89">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A90">
-        <v>89</v>
-      </c>
-      <c r="B90" t="s">
-        <v>471</v>
-      </c>
-      <c r="C90">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A91">
-        <v>90</v>
-      </c>
-      <c r="B91" t="s">
-        <v>429</v>
-      </c>
-      <c r="C91">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A92">
-        <v>91</v>
-      </c>
-      <c r="B92" t="s">
-        <v>472</v>
-      </c>
-      <c r="C92">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A93">
-        <v>92</v>
-      </c>
-      <c r="B93" t="s">
-        <v>473</v>
-      </c>
-      <c r="C93">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A94">
-        <v>93</v>
-      </c>
-      <c r="B94" t="s">
-        <v>474</v>
-      </c>
-      <c r="C94">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A95">
-        <v>94</v>
-      </c>
-      <c r="B95" t="s">
-        <v>475</v>
-      </c>
-      <c r="C95">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A96">
-        <v>95</v>
-      </c>
-      <c r="B96" t="s">
-        <v>476</v>
-      </c>
-      <c r="C96">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A97">
-        <v>96</v>
-      </c>
-      <c r="B97" t="s">
-        <v>477</v>
-      </c>
-      <c r="C97">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A98">
-        <v>97</v>
-      </c>
-      <c r="B98" t="s">
-        <v>478</v>
-      </c>
-      <c r="C98">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A99">
-        <v>98</v>
-      </c>
-      <c r="B99" t="s">
-        <v>479</v>
-      </c>
-      <c r="C99">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A100">
-        <v>99</v>
-      </c>
-      <c r="B100" t="s">
-        <v>480</v>
-      </c>
-      <c r="C100">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A101">
-        <v>100</v>
-      </c>
-      <c r="B101" t="s">
-        <v>481</v>
-      </c>
-      <c r="C101">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A102">
-        <v>101</v>
-      </c>
-      <c r="B102" t="s">
-        <v>482</v>
-      </c>
-      <c r="C102">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A103">
-        <v>102</v>
-      </c>
-      <c r="B103" t="s">
-        <v>415</v>
-      </c>
-      <c r="C103">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A104">
-        <v>103</v>
-      </c>
-      <c r="B104" t="s">
-        <v>483</v>
-      </c>
-      <c r="C104">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A105">
-        <v>104</v>
-      </c>
-      <c r="B105" t="s">
-        <v>484</v>
-      </c>
-      <c r="C105">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A106">
-        <v>105</v>
-      </c>
-      <c r="B106" t="s">
-        <v>459</v>
-      </c>
-      <c r="C106">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A107">
-        <v>106</v>
-      </c>
-      <c r="B107" t="s">
-        <v>485</v>
-      </c>
-      <c r="C107">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A108">
-        <v>107</v>
-      </c>
-      <c r="B108" t="s">
-        <v>486</v>
-      </c>
-      <c r="C108">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A109">
-        <v>108</v>
-      </c>
-      <c r="B109" t="s">
-        <v>441</v>
-      </c>
-      <c r="C109">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A110">
-        <v>109</v>
-      </c>
-      <c r="B110" t="s">
-        <v>487</v>
-      </c>
-      <c r="C110">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A111">
-        <v>110</v>
-      </c>
-      <c r="B111" t="s">
-        <v>488</v>
-      </c>
-      <c r="C111">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A112">
-        <v>111</v>
-      </c>
-      <c r="B112" t="s">
-        <v>489</v>
-      </c>
-      <c r="C112">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A113">
-        <v>112</v>
-      </c>
-      <c r="B113" t="s">
-        <v>462</v>
-      </c>
-      <c r="C113">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A114">
-        <v>113</v>
-      </c>
-      <c r="B114" t="s">
-        <v>447</v>
-      </c>
-      <c r="C114">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A115">
-        <v>114</v>
-      </c>
-      <c r="B115" t="s">
-        <v>490</v>
-      </c>
-      <c r="C115">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A116">
-        <v>115</v>
-      </c>
-      <c r="B116" t="s">
-        <v>491</v>
-      </c>
-      <c r="C116">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A117">
-        <v>116</v>
-      </c>
-      <c r="B117" t="s">
-        <v>492</v>
-      </c>
-      <c r="C117">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A118">
-        <v>117</v>
-      </c>
-      <c r="B118" t="s">
-        <v>422</v>
-      </c>
-      <c r="C118">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A119">
-        <v>118</v>
-      </c>
-      <c r="B119" t="s">
-        <v>493</v>
-      </c>
-      <c r="C119">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A120">
-        <v>119</v>
-      </c>
-      <c r="B120" t="s">
-        <v>435</v>
-      </c>
-      <c r="C120">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A121">
-        <v>120</v>
-      </c>
-      <c r="B121" t="s">
-        <v>494</v>
-      </c>
-      <c r="C121">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A122">
-        <v>121</v>
-      </c>
-      <c r="B122" t="s">
-        <v>495</v>
-      </c>
-      <c r="C122">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A123">
-        <v>122</v>
-      </c>
-      <c r="B123" t="s">
-        <v>457</v>
-      </c>
-      <c r="C123">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A124">
-        <v>123</v>
-      </c>
-      <c r="B124" t="s">
-        <v>399</v>
-      </c>
-      <c r="C124">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A125">
-        <v>124</v>
-      </c>
-      <c r="B125" t="s">
-        <v>428</v>
-      </c>
-      <c r="C125">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A126">
-        <v>125</v>
-      </c>
-      <c r="B126" t="s">
-        <v>496</v>
-      </c>
-      <c r="C126">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A127">
-        <v>126</v>
-      </c>
-      <c r="B127" t="s">
-        <v>401</v>
-      </c>
-      <c r="C127">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A128">
-        <v>127</v>
-      </c>
-      <c r="B128" t="s">
-        <v>497</v>
-      </c>
-      <c r="C128">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A129">
-        <v>128</v>
-      </c>
-      <c r="B129" t="s">
-        <v>467</v>
-      </c>
-      <c r="C129">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A130">
-        <v>129</v>
-      </c>
-      <c r="B130" t="s">
-        <v>420</v>
-      </c>
-      <c r="C130">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A131">
-        <v>130</v>
-      </c>
-      <c r="B131" t="s">
-        <v>498</v>
-      </c>
-      <c r="C131">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A132">
-        <v>131</v>
-      </c>
-      <c r="B132" t="s">
-        <v>433</v>
-      </c>
-      <c r="C132">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A133">
-        <v>132</v>
-      </c>
-      <c r="B133" t="s">
-        <v>408</v>
-      </c>
-      <c r="C133">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A134">
-        <v>133</v>
-      </c>
-      <c r="B134" t="s">
-        <v>499</v>
-      </c>
-      <c r="C134">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A135">
-        <v>134</v>
-      </c>
-      <c r="B135" t="s">
-        <v>430</v>
-      </c>
-      <c r="C135">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A136">
-        <v>135</v>
-      </c>
-      <c r="B136" t="s">
-        <v>429</v>
-      </c>
-      <c r="C136">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A137">
-        <v>136</v>
-      </c>
-      <c r="B137" t="s">
-        <v>415</v>
-      </c>
-      <c r="C137">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A138">
-        <v>137</v>
-      </c>
-      <c r="B138" t="s">
-        <v>487</v>
-      </c>
-      <c r="C138">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A139">
-        <v>138</v>
-      </c>
-      <c r="B139" t="s">
-        <v>500</v>
-      </c>
-      <c r="C139">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A140">
-        <v>139</v>
-      </c>
-      <c r="B140" t="s">
-        <v>501</v>
-      </c>
-      <c r="C140">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A141">
-        <v>140</v>
-      </c>
-      <c r="B141" t="s">
-        <v>422</v>
-      </c>
-      <c r="C141">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A142">
-        <v>141</v>
-      </c>
-      <c r="B142" t="s">
-        <v>459</v>
-      </c>
-      <c r="C142">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A143">
-        <v>142</v>
-      </c>
-      <c r="B143" t="s">
-        <v>502</v>
-      </c>
-      <c r="C143">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A144">
-        <v>143</v>
-      </c>
-      <c r="B144" t="s">
-        <v>503</v>
-      </c>
-      <c r="C144">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A145">
-        <v>144</v>
-      </c>
-      <c r="B145" t="s">
-        <v>504</v>
-      </c>
-      <c r="C145">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A146">
-        <v>145</v>
-      </c>
-      <c r="B146" t="s">
-        <v>477</v>
-      </c>
-      <c r="C146">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A147">
-        <v>146</v>
-      </c>
-      <c r="B147" t="s">
-        <v>445</v>
-      </c>
-      <c r="C147">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A148">
-        <v>147</v>
-      </c>
-      <c r="B148" t="s">
-        <v>435</v>
-      </c>
-      <c r="C148">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A149">
-        <v>148</v>
-      </c>
-      <c r="B149" t="s">
-        <v>505</v>
-      </c>
-      <c r="C149">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A150">
-        <v>149</v>
-      </c>
-      <c r="B150" t="s">
-        <v>506</v>
-      </c>
-      <c r="C150">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A151">
-        <v>150</v>
-      </c>
-      <c r="B151" t="s">
-        <v>462</v>
-      </c>
-      <c r="C151">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A152">
-        <v>151</v>
-      </c>
-      <c r="B152" t="s">
-        <v>507</v>
-      </c>
-      <c r="C152">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A153">
-        <v>152</v>
-      </c>
-      <c r="B153" t="s">
-        <v>440</v>
-      </c>
-      <c r="C153">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A154">
-        <v>153</v>
-      </c>
-      <c r="B154" t="s">
-        <v>447</v>
-      </c>
-      <c r="C154">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A155">
-        <v>154</v>
-      </c>
-      <c r="B155" t="s">
-        <v>508</v>
-      </c>
-      <c r="C155">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A156">
-        <v>155</v>
-      </c>
-      <c r="B156" t="s">
-        <v>422</v>
-      </c>
-      <c r="C156">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A157">
-        <v>156</v>
-      </c>
-      <c r="B157" t="s">
-        <v>464</v>
-      </c>
-      <c r="C157">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A158">
-        <v>157</v>
-      </c>
-      <c r="B158" t="s">
-        <v>509</v>
-      </c>
-      <c r="C158">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A159">
-        <v>158</v>
-      </c>
-      <c r="B159" t="s">
-        <v>474</v>
-      </c>
-      <c r="C159">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A160">
-        <v>159</v>
-      </c>
-      <c r="B160" t="s">
-        <v>415</v>
-      </c>
-      <c r="C160">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A161">
-        <v>160</v>
-      </c>
-      <c r="B161" t="s">
-        <v>438</v>
-      </c>
-      <c r="C161">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A162">
-        <v>161</v>
-      </c>
-      <c r="B162" t="s">
-        <v>510</v>
-      </c>
-      <c r="C162">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A163">
-        <v>162</v>
-      </c>
-      <c r="B163" t="s">
-        <v>511</v>
-      </c>
-      <c r="C163">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A164">
-        <v>163</v>
-      </c>
-      <c r="B164" t="s">
-        <v>476</v>
-      </c>
-      <c r="C164">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A165">
-        <v>164</v>
-      </c>
-      <c r="B165" t="s">
-        <v>457</v>
-      </c>
-      <c r="C165">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A166">
-        <v>165</v>
-      </c>
-      <c r="B166" t="s">
-        <v>420</v>
-      </c>
-      <c r="C166">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A167">
-        <v>166</v>
-      </c>
-      <c r="B167" t="s">
-        <v>453</v>
-      </c>
-      <c r="C167">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A168">
-        <v>167</v>
-      </c>
-      <c r="B168" t="s">
-        <v>512</v>
-      </c>
-      <c r="C168">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A169">
-        <v>168</v>
-      </c>
-      <c r="B169" t="s">
-        <v>441</v>
-      </c>
-      <c r="C169">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A170">
-        <v>169</v>
-      </c>
-      <c r="B170" t="s">
-        <v>460</v>
-      </c>
-      <c r="C170">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A171">
-        <v>170</v>
-      </c>
-      <c r="B171" t="s">
-        <v>429</v>
-      </c>
-      <c r="C171">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A172">
-        <v>171</v>
-      </c>
-      <c r="B172" t="s">
-        <v>467</v>
-      </c>
-      <c r="C172">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A173">
-        <v>172</v>
-      </c>
-      <c r="B173" t="s">
-        <v>462</v>
-      </c>
-      <c r="C173">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A174">
-        <v>173</v>
-      </c>
-      <c r="B174" t="s">
-        <v>390</v>
-      </c>
-      <c r="C174">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A175">
-        <v>174</v>
-      </c>
-      <c r="B175" t="s">
-        <v>459</v>
-      </c>
-      <c r="C175">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A176">
-        <v>175</v>
-      </c>
-      <c r="B176" t="s">
-        <v>416</v>
-      </c>
-      <c r="C176">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A177">
-        <v>176</v>
-      </c>
-      <c r="B177" t="s">
-        <v>469</v>
-      </c>
-      <c r="C177">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A178">
-        <v>177</v>
-      </c>
-      <c r="B178" t="s">
-        <v>401</v>
-      </c>
-      <c r="C178">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A179">
-        <v>178</v>
-      </c>
-      <c r="B179" t="s">
-        <v>403</v>
-      </c>
-      <c r="C179">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A180">
-        <v>179</v>
-      </c>
-      <c r="B180" t="s">
-        <v>493</v>
-      </c>
-      <c r="C180">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A181">
-        <v>180</v>
-      </c>
-      <c r="B181" t="s">
-        <v>494</v>
-      </c>
-      <c r="C181">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A182">
-        <v>181</v>
-      </c>
-      <c r="B182" t="s">
-        <v>458</v>
-      </c>
-      <c r="C182">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A183">
-        <v>182</v>
-      </c>
-      <c r="B183" t="s">
-        <v>422</v>
-      </c>
-      <c r="C183">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A184">
-        <v>183</v>
-      </c>
-      <c r="B184" t="s">
-        <v>426</v>
-      </c>
-      <c r="C184">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A185">
-        <v>184</v>
-      </c>
-      <c r="B185" t="s">
-        <v>399</v>
-      </c>
-      <c r="C185">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A186">
-        <v>185</v>
-      </c>
-      <c r="B186" t="s">
-        <v>442</v>
-      </c>
-      <c r="C186">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A187">
-        <v>186</v>
-      </c>
-      <c r="B187" t="s">
-        <v>513</v>
-      </c>
-      <c r="C187">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A188">
-        <v>187</v>
-      </c>
-      <c r="B188" t="s">
-        <v>408</v>
-      </c>
-      <c r="C188">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A189">
-        <v>188</v>
-      </c>
-      <c r="B189" t="s">
-        <v>478</v>
-      </c>
-      <c r="C189">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A190">
-        <v>189</v>
-      </c>
-      <c r="B190" t="s">
-        <v>447</v>
-      </c>
-      <c r="C190">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A191">
-        <v>190</v>
-      </c>
-      <c r="B191" t="s">
-        <v>455</v>
-      </c>
-      <c r="C191">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A192">
-        <v>191</v>
-      </c>
-      <c r="B192" t="s">
-        <v>387</v>
-      </c>
-      <c r="C192">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A193">
-        <v>192</v>
-      </c>
-      <c r="B193" t="s">
-        <v>415</v>
-      </c>
-      <c r="C193">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A194">
-        <v>193</v>
-      </c>
-      <c r="B194" t="s">
-        <v>430</v>
-      </c>
-      <c r="C194">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A195">
-        <v>194</v>
-      </c>
-      <c r="B195" t="s">
-        <v>466</v>
-      </c>
-      <c r="C195">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A196">
-        <v>195</v>
-      </c>
-      <c r="B196" t="s">
-        <v>433</v>
-      </c>
-      <c r="C196">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A197">
-        <v>196</v>
-      </c>
-      <c r="B197" t="s">
-        <v>477</v>
-      </c>
-      <c r="C197">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A198">
-        <v>197</v>
-      </c>
-      <c r="B198" t="s">
-        <v>514</v>
-      </c>
-      <c r="C198">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A199">
-        <v>198</v>
-      </c>
-      <c r="B199" t="s">
-        <v>487</v>
-      </c>
-      <c r="C199">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A200">
-        <v>199</v>
-      </c>
-      <c r="B200" t="s">
-        <v>429</v>
-      </c>
-      <c r="C200">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A201">
-        <v>200</v>
-      </c>
-      <c r="B201" t="s">
-        <v>401</v>
-      </c>
-      <c r="C201">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B401">
-    <sortCondition ref="A2:A401"/>
-  </sortState>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>